<commit_message>
added a Collections page
filter by collection -- involves a new row in CSV/XLSX, new View, new page layout (Collections List)
</commit_message>
<xml_diff>
--- a/dist/catalog.xlsx
+++ b/dist/catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/astrid/GitHub/personal-portfolio/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9415CD1-9542-D346-9AEF-D71DC85F45DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB63AAEB-F5E8-B049-8093-B5B327714203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="18480" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="69">
   <si>
     <t>file</t>
   </si>
@@ -209,6 +209,24 @@
   </si>
   <si>
     <t>tooplate-exhibit-09.jpg</t>
+  </si>
+  <si>
+    <t>collections</t>
+  </si>
+  <si>
+    <t>[Spring]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Fall], [Landscape] </t>
+  </si>
+  <si>
+    <t>[Landscape], [Spring]</t>
+  </si>
+  <si>
+    <t>[Landscape]</t>
+  </si>
+  <si>
+    <t>[other]</t>
   </si>
 </sst>
 </file>
@@ -591,7 +609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
@@ -602,7 +620,7 @@
     <col min="7" max="7" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -624,8 +642,11 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -644,8 +665,11 @@
       <c r="F2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -665,7 +689,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -684,8 +708,11 @@
       <c r="F4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -705,7 +732,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>48</v>
       </c>
@@ -725,7 +752,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -745,7 +772,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>50</v>
       </c>
@@ -765,7 +792,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>51</v>
       </c>
@@ -785,7 +812,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>52</v>
       </c>
@@ -805,7 +832,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>53</v>
       </c>
@@ -824,8 +851,11 @@
       <c r="F11" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -845,7 +875,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -865,7 +895,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>56</v>
       </c>
@@ -884,8 +914,11 @@
       <c r="F14" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -905,7 +938,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>58</v>
       </c>
@@ -925,7 +958,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -944,8 +977,11 @@
       <c r="F17" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="H17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -964,8 +1000,11 @@
       <c r="F18" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="H18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>61</v>
       </c>
@@ -985,7 +1024,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>62</v>
       </c>

</xml_diff>

<commit_message>
upgrading formatting, added work previews on collections list
</commit_message>
<xml_diff>
--- a/dist/catalog.xlsx
+++ b/dist/catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/astrid/GitHub/personal-portfolio/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB63AAEB-F5E8-B049-8093-B5B327714203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47AE6331-2BB2-A349-8490-A7E52CD72B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="18480" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="73">
   <si>
     <t>file</t>
   </si>
@@ -227,6 +227,18 @@
   </si>
   <si>
     <t>[other]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[this], [there], [apple], [banana], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">[other], [together], [paint], [sketch], [gesso], </t>
+  </si>
+  <si>
+    <t>[more], [less]</t>
+  </si>
+  <si>
+    <t>[more]</t>
   </si>
 </sst>
 </file>
@@ -751,6 +763,9 @@
       <c r="F6" t="s">
         <v>21</v>
       </c>
+      <c r="H6" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -771,6 +786,9 @@
       <c r="F7" t="s">
         <v>24</v>
       </c>
+      <c r="H7" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -791,6 +809,9 @@
       <c r="F8" t="s">
         <v>27</v>
       </c>
+      <c r="H8" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -1023,6 +1044,9 @@
       <c r="F19" t="s">
         <v>42</v>
       </c>
+      <c r="H19" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
@@ -1042,6 +1066,9 @@
       </c>
       <c r="F20" t="s">
         <v>43</v>
+      </c>
+      <c r="H20" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>